<commit_message>
Include part numbers that sit below the QTY block on the D sheet
Simplify extraction to one rule: a cell counts as a genuine batches-
per-day entry only when it's a literal number, not a formula. This
still captures every QTY-block part row (687/D) and every flat Rest-
sheet row as before, but also now picks up the part numbers further
down the D sheet (e.g. rows 33+) that hold plain typed-in values with
no QTY row underneath -- these were previously skipped entirely.

QTY rows, Total/Non-687 footers, and subtotal rows are all formulas,
so they keep getting excluded automatically without needing separate
label-matching logic.

Regenerated CategorySIPMaintain.7.30.long.xlsx: 86 rows across 15
part numbers (up from 75/13, now including T521D686M025ATE0707652
and T521D157M016ATE050).
</commit_message>
<xml_diff>
--- a/CategorySIPMaintain.7.30.long.xlsx
+++ b/CategorySIPMaintain.7.30.long.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1572,39 +1572,39 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>T530X158M2R5ATE005</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="n">
-        <v>46235</v>
-      </c>
-      <c r="D63" s="2" t="n">
-        <v>5</v>
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>T521D686M025ATE0707652</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>T530X158M2R5ATE005</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="n">
-        <v>46236</v>
-      </c>
-      <c r="D64" s="2" t="n">
-        <v>5</v>
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>T521D686M025ATE0707652</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="65">
@@ -1615,14 +1615,14 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>T530X158M2R5ATE005</t>
+          <t>T521D157M016ATE050</t>
         </is>
       </c>
       <c r="C65" s="5" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="D65" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66">
@@ -1633,50 +1633,50 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>T530X158M2R5ATE005</t>
+          <t>T521D157M016ATE050</t>
         </is>
       </c>
       <c r="C66" s="5" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="D66" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>T530X158M2R5ATE005</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D67" s="4" t="n">
-        <v>5</v>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>T598D336M025ATE060</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>T530X158M2R5ATE005</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="n">
-        <v>46240</v>
-      </c>
-      <c r="D68" s="4" t="n">
-        <v>5</v>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>T598D336M025ATE060</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -1687,50 +1687,50 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>T530X158M2R5ATE005</t>
+          <t>T598D336M025ATE060</t>
         </is>
       </c>
       <c r="C69" s="5" t="n">
-        <v>46241</v>
+        <v>46237</v>
       </c>
       <c r="D69" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>T520V477M2R5ATE018</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="n">
-        <v>46235</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>2</v>
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>T598D336M025ATE060</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>T520V477M2R5ATE018</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="n">
-        <v>46236</v>
-      </c>
-      <c r="D71" s="2" t="n">
-        <v>2</v>
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>T598D336M025ATE060</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -1741,14 +1741,14 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>T520V477M2R5ATE018</t>
+          <t>T598D336M025ATE060</t>
         </is>
       </c>
       <c r="C72" s="5" t="n">
-        <v>46237</v>
+        <v>46240</v>
       </c>
       <c r="D72" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -1759,50 +1759,50 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>T520V477M2R5ATE018</t>
+          <t>T598D336M025ATE060</t>
         </is>
       </c>
       <c r="C73" s="5" t="n">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="D73" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>T520V477M2R5ATE018</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D74" s="4" t="n">
-        <v>2</v>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>T520V477M2R5ATE018</t>
-        </is>
-      </c>
-      <c r="C75" s="5" t="n">
-        <v>46240</v>
-      </c>
-      <c r="D75" s="4" t="n">
-        <v>2</v>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="76">
@@ -1813,13 +1813,211 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D78" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>T530X158M2R5ATE005</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>46241</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
           <t>T520V477M2R5ATE018</t>
         </is>
       </c>
-      <c r="C76" s="5" t="n">
+      <c r="C81" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>46236</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="n">
+        <v>46238</v>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>46240</v>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>T520V477M2R5ATE018</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="n">
         <v>46241</v>
       </c>
-      <c r="D76" s="4" t="n">
+      <c r="D87" s="4" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>